<commit_message>
update figures, add czech descriptions, change colours
</commit_message>
<xml_diff>
--- a/Outputs/Tables/model_results.xlsx
+++ b/Outputs/Tables/model_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1346" uniqueCount="169">
   <si>
     <t>model_id</t>
   </si>
@@ -458,6 +458,69 @@
   </si>
   <si>
     <t>H10_H11_dens_sel</t>
+  </si>
+  <si>
+    <t>H7_spont</t>
+  </si>
+  <si>
+    <t>subset</t>
+  </si>
+  <si>
+    <t>Spontaneous count, visit 1</t>
+  </si>
+  <si>
+    <t>H7_prov</t>
+  </si>
+  <si>
+    <t>H8_spont</t>
+  </si>
+  <si>
+    <t>Spontaneous count, visit 2</t>
+  </si>
+  <si>
+    <t>H8_prov</t>
+  </si>
+  <si>
+    <t>H9_v1_class</t>
+  </si>
+  <si>
+    <t>loudness_class80-90</t>
+  </si>
+  <si>
+    <t>Device loudness 80–90 dB (vs &lt; 80 dB)</t>
+  </si>
+  <si>
+    <t>devices of 80–90 dB</t>
+  </si>
+  <si>
+    <t>vs &lt; 80 dB</t>
+  </si>
+  <si>
+    <t>loudness_class90-100</t>
+  </si>
+  <si>
+    <t>Device loudness 90–100 dB (vs &lt; 80 dB)</t>
+  </si>
+  <si>
+    <t>devices of 90–100 dB</t>
+  </si>
+  <si>
+    <t>loudness_class&gt;=100</t>
+  </si>
+  <si>
+    <t>Device loudness ≥ 100 dB (vs &lt; 80 dB)</t>
+  </si>
+  <si>
+    <t>devices of 100 dB or more</t>
+  </si>
+  <si>
+    <t>H9_v2_class</t>
+  </si>
+  <si>
+    <t>H10_H11_dens_selonly</t>
+  </si>
+  <si>
+    <t>H10_H11_dens_selonly_lowcal</t>
   </si>
 </sst>
 </file>
@@ -800,7 +863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AM85"/>
+  <dimension ref="A1:AM109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:39" s="1" customFormat="1">
@@ -10144,6 +10207,2424 @@
         <v>0.8228564066085329</v>
       </c>
     </row>
+    <row r="86" spans="1:39">
+      <c r="A86" t="s">
+        <v>148</v>
+      </c>
+      <c r="B86" t="s">
+        <v>77</v>
+      </c>
+      <c r="C86" t="s">
+        <v>149</v>
+      </c>
+      <c r="D86" t="s">
+        <v>41</v>
+      </c>
+      <c r="E86" t="b">
+        <v>1</v>
+      </c>
+      <c r="F86" t="s">
+        <v>150</v>
+      </c>
+      <c r="G86" t="s">
+        <v>43</v>
+      </c>
+      <c r="H86">
+        <v>362</v>
+      </c>
+      <c r="I86" t="s">
+        <v>79</v>
+      </c>
+      <c r="J86" t="s">
+        <v>80</v>
+      </c>
+      <c r="K86" t="s">
+        <v>81</v>
+      </c>
+      <c r="L86" t="s">
+        <v>82</v>
+      </c>
+      <c r="M86">
+        <v>-0.2088554237632885</v>
+      </c>
+      <c r="N86">
+        <v>0.09779084741077615</v>
+      </c>
+      <c r="O86">
+        <v>-0.4005219627060618</v>
+      </c>
+      <c r="P86">
+        <v>-0.01718888482051531</v>
+      </c>
+      <c r="Q86" t="s">
+        <v>48</v>
+      </c>
+      <c r="R86">
+        <v>0.8115125525934835</v>
+      </c>
+      <c r="S86">
+        <v>0.6699702552672927</v>
+      </c>
+      <c r="T86">
+        <v>0.9829580012534348</v>
+      </c>
+      <c r="U86">
+        <v>-2.135735902624702</v>
+      </c>
+      <c r="V86">
+        <v>0.03270094625792737</v>
+      </c>
+      <c r="W86" t="s">
+        <v>83</v>
+      </c>
+      <c r="X86" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y86">
+        <v>0.4178054304821218</v>
+      </c>
+      <c r="Z86">
+        <v>343.6368381376739</v>
+      </c>
+      <c r="AA86">
+        <v>0.01348136608387085</v>
+      </c>
+      <c r="AD86">
+        <v>-0.01692473162528257</v>
+      </c>
+      <c r="AE86">
+        <v>0.7244576351878997</v>
+      </c>
+      <c r="AF86">
+        <v>-0.0343128220471781</v>
+      </c>
+      <c r="AG86">
+        <v>0.746210819363994</v>
+      </c>
+      <c r="AH86">
+        <v>0.9965384836384295</v>
+      </c>
+    </row>
+    <row r="87" spans="1:39">
+      <c r="A87" t="s">
+        <v>151</v>
+      </c>
+      <c r="B87" t="s">
+        <v>77</v>
+      </c>
+      <c r="C87" t="s">
+        <v>149</v>
+      </c>
+      <c r="D87" t="s">
+        <v>41</v>
+      </c>
+      <c r="E87" t="b">
+        <v>0</v>
+      </c>
+      <c r="F87" t="s">
+        <v>101</v>
+      </c>
+      <c r="G87" t="s">
+        <v>43</v>
+      </c>
+      <c r="H87">
+        <v>361</v>
+      </c>
+      <c r="I87" t="s">
+        <v>79</v>
+      </c>
+      <c r="J87" t="s">
+        <v>80</v>
+      </c>
+      <c r="K87" t="s">
+        <v>81</v>
+      </c>
+      <c r="L87" t="s">
+        <v>82</v>
+      </c>
+      <c r="M87">
+        <v>-0.2552815108724086</v>
+      </c>
+      <c r="N87">
+        <v>0.0690673713296034</v>
+      </c>
+      <c r="O87">
+        <v>-0.3906510711852856</v>
+      </c>
+      <c r="P87">
+        <v>-0.1199119505595317</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>48</v>
+      </c>
+      <c r="R87">
+        <v>0.7746983812442502</v>
+      </c>
+      <c r="S87">
+        <v>0.6766162057453095</v>
+      </c>
+      <c r="T87">
+        <v>0.8869985330034671</v>
+      </c>
+      <c r="U87">
+        <v>-3.696123161458598</v>
+      </c>
+      <c r="V87">
+        <v>0.0002189168032810251</v>
+      </c>
+      <c r="W87" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y87">
+        <v>0.8073246442375696</v>
+      </c>
+      <c r="Z87">
+        <v>605.4003700524531</v>
+      </c>
+      <c r="AA87">
+        <v>0.02281027888795328</v>
+      </c>
+      <c r="AD87">
+        <v>0.04380605359686635</v>
+      </c>
+      <c r="AE87">
+        <v>0.02503613505867666</v>
+      </c>
+      <c r="AF87">
+        <v>0.07946400378379827</v>
+      </c>
+      <c r="AG87">
+        <v>0.03944389615720765</v>
+      </c>
+      <c r="AH87">
+        <v>0.0002702145147677193</v>
+      </c>
+      <c r="AI87">
+        <v>-0.02462231244713045</v>
+      </c>
+      <c r="AJ87">
+        <v>0.8208617609151636</v>
+      </c>
+      <c r="AK87">
+        <v>0.01287173401239563</v>
+      </c>
+      <c r="AL87">
+        <v>0.3668818456876382</v>
+      </c>
+      <c r="AM87">
+        <v>0.640289330391089</v>
+      </c>
+    </row>
+    <row r="88" spans="1:39">
+      <c r="A88" t="s">
+        <v>151</v>
+      </c>
+      <c r="B88" t="s">
+        <v>77</v>
+      </c>
+      <c r="C88" t="s">
+        <v>149</v>
+      </c>
+      <c r="D88" t="s">
+        <v>50</v>
+      </c>
+      <c r="E88" t="b">
+        <v>1</v>
+      </c>
+      <c r="F88" t="s">
+        <v>101</v>
+      </c>
+      <c r="G88" t="s">
+        <v>133</v>
+      </c>
+      <c r="H88">
+        <v>361</v>
+      </c>
+      <c r="I88" t="s">
+        <v>79</v>
+      </c>
+      <c r="J88" t="s">
+        <v>80</v>
+      </c>
+      <c r="K88" t="s">
+        <v>81</v>
+      </c>
+      <c r="L88" t="s">
+        <v>82</v>
+      </c>
+      <c r="M88">
+        <v>-0.2805661320636845</v>
+      </c>
+      <c r="N88">
+        <v>0.06846467710639124</v>
+      </c>
+      <c r="O88">
+        <v>-0.4147544334053753</v>
+      </c>
+      <c r="P88">
+        <v>-0.1463778307219938</v>
+      </c>
+      <c r="Q88" t="s">
+        <v>48</v>
+      </c>
+      <c r="R88">
+        <v>0.7553559891400513</v>
+      </c>
+      <c r="S88">
+        <v>0.6605024581308733</v>
+      </c>
+      <c r="T88">
+        <v>0.8638312595298364</v>
+      </c>
+      <c r="U88">
+        <v>-4.097969112272252</v>
+      </c>
+      <c r="V88">
+        <v>4.167908803745006E-05</v>
+      </c>
+      <c r="W88" t="s">
+        <v>83</v>
+      </c>
+      <c r="X88" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y88">
+        <v>0.8073246442375696</v>
+      </c>
+      <c r="Z88">
+        <v>587.6867960920654</v>
+      </c>
+      <c r="AA88">
+        <v>0.02677289318673459</v>
+      </c>
+      <c r="AB88">
+        <v>260.135697419514</v>
+      </c>
+      <c r="AC88">
+        <v>0.8121735641837692</v>
+      </c>
+      <c r="AD88">
+        <v>0.04380605359686635</v>
+      </c>
+      <c r="AE88">
+        <v>0.02503613505867666</v>
+      </c>
+      <c r="AF88">
+        <v>0.07946400378379827</v>
+      </c>
+      <c r="AG88">
+        <v>0.03944389615720765</v>
+      </c>
+      <c r="AH88">
+        <v>0.0002702145147677193</v>
+      </c>
+      <c r="AI88">
+        <v>-0.02462231244713045</v>
+      </c>
+      <c r="AJ88">
+        <v>0.8208617609151636</v>
+      </c>
+      <c r="AK88">
+        <v>0.01287173401239563</v>
+      </c>
+      <c r="AL88">
+        <v>0.3668818456876382</v>
+      </c>
+      <c r="AM88">
+        <v>0.640289330391089</v>
+      </c>
+    </row>
+    <row r="89" spans="1:39">
+      <c r="A89" t="s">
+        <v>152</v>
+      </c>
+      <c r="B89" t="s">
+        <v>85</v>
+      </c>
+      <c r="C89" t="s">
+        <v>149</v>
+      </c>
+      <c r="D89" t="s">
+        <v>41</v>
+      </c>
+      <c r="E89" t="b">
+        <v>1</v>
+      </c>
+      <c r="F89" t="s">
+        <v>153</v>
+      </c>
+      <c r="G89" t="s">
+        <v>43</v>
+      </c>
+      <c r="H89">
+        <v>354</v>
+      </c>
+      <c r="I89" t="s">
+        <v>87</v>
+      </c>
+      <c r="J89" t="s">
+        <v>88</v>
+      </c>
+      <c r="K89" t="s">
+        <v>89</v>
+      </c>
+      <c r="L89" t="s">
+        <v>82</v>
+      </c>
+      <c r="M89">
+        <v>0.2278021706401877</v>
+      </c>
+      <c r="N89">
+        <v>0.1185035248746196</v>
+      </c>
+      <c r="O89">
+        <v>-0.004460470155113139</v>
+      </c>
+      <c r="P89">
+        <v>0.4600648114354884</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>48</v>
+      </c>
+      <c r="R89">
+        <v>1.255836859454287</v>
+      </c>
+      <c r="S89">
+        <v>0.9955494629676021</v>
+      </c>
+      <c r="T89">
+        <v>1.58417665443041</v>
+      </c>
+      <c r="U89">
+        <v>1.922324005815096</v>
+      </c>
+      <c r="V89">
+        <v>0.05456500119478824</v>
+      </c>
+      <c r="W89" t="s">
+        <v>83</v>
+      </c>
+      <c r="X89" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y89">
+        <v>0.5811539804444464</v>
+      </c>
+      <c r="Z89">
+        <v>331.9086412875165</v>
+      </c>
+      <c r="AA89">
+        <v>0.03099809921225616</v>
+      </c>
+      <c r="AD89">
+        <v>-0.01962586642447821</v>
+      </c>
+      <c r="AE89">
+        <v>0.757921675728828</v>
+      </c>
+      <c r="AF89">
+        <v>0.02310477793664775</v>
+      </c>
+      <c r="AG89">
+        <v>0.2889220518073117</v>
+      </c>
+      <c r="AH89">
+        <v>0.7680579011322347</v>
+      </c>
+    </row>
+    <row r="90" spans="1:39">
+      <c r="A90" t="s">
+        <v>152</v>
+      </c>
+      <c r="B90" t="s">
+        <v>90</v>
+      </c>
+      <c r="C90" t="s">
+        <v>149</v>
+      </c>
+      <c r="D90" t="s">
+        <v>41</v>
+      </c>
+      <c r="E90" t="b">
+        <v>1</v>
+      </c>
+      <c r="F90" t="s">
+        <v>153</v>
+      </c>
+      <c r="G90" t="s">
+        <v>43</v>
+      </c>
+      <c r="H90">
+        <v>354</v>
+      </c>
+      <c r="I90" t="s">
+        <v>91</v>
+      </c>
+      <c r="J90" t="s">
+        <v>92</v>
+      </c>
+      <c r="K90" t="s">
+        <v>93</v>
+      </c>
+      <c r="L90" t="s">
+        <v>94</v>
+      </c>
+      <c r="M90">
+        <v>-0.8897890231459847</v>
+      </c>
+      <c r="N90">
+        <v>0.4431778711812006</v>
+      </c>
+      <c r="O90">
+        <v>-1.758401689406269</v>
+      </c>
+      <c r="P90">
+        <v>-0.02117635688570019</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>48</v>
+      </c>
+      <c r="R90">
+        <v>0.4107424007511841</v>
+      </c>
+      <c r="S90">
+        <v>0.1723200648212456</v>
+      </c>
+      <c r="T90">
+        <v>0.9790462877892667</v>
+      </c>
+      <c r="U90">
+        <v>-2.007746958968039</v>
+      </c>
+      <c r="V90">
+        <v>0.04467018779808658</v>
+      </c>
+      <c r="Y90">
+        <v>0.5811539804444464</v>
+      </c>
+      <c r="Z90">
+        <v>331.9086412875165</v>
+      </c>
+      <c r="AA90">
+        <v>0.03099809921225616</v>
+      </c>
+      <c r="AD90">
+        <v>-0.01962586642447821</v>
+      </c>
+      <c r="AE90">
+        <v>0.757921675728828</v>
+      </c>
+      <c r="AF90">
+        <v>0.02310477793664775</v>
+      </c>
+      <c r="AG90">
+        <v>0.2889220518073117</v>
+      </c>
+      <c r="AH90">
+        <v>0.7680579011322347</v>
+      </c>
+    </row>
+    <row r="91" spans="1:39">
+      <c r="A91" t="s">
+        <v>152</v>
+      </c>
+      <c r="B91" t="s">
+        <v>90</v>
+      </c>
+      <c r="C91" t="s">
+        <v>149</v>
+      </c>
+      <c r="D91" t="s">
+        <v>41</v>
+      </c>
+      <c r="E91" t="b">
+        <v>1</v>
+      </c>
+      <c r="F91" t="s">
+        <v>153</v>
+      </c>
+      <c r="G91" t="s">
+        <v>43</v>
+      </c>
+      <c r="H91">
+        <v>354</v>
+      </c>
+      <c r="I91" t="s">
+        <v>95</v>
+      </c>
+      <c r="J91" t="s">
+        <v>96</v>
+      </c>
+      <c r="K91" t="s">
+        <v>97</v>
+      </c>
+      <c r="L91" t="s">
+        <v>94</v>
+      </c>
+      <c r="M91">
+        <v>1.196772725503205</v>
+      </c>
+      <c r="N91">
+        <v>0.78141282463241</v>
+      </c>
+      <c r="O91">
+        <v>-0.3347682678340311</v>
+      </c>
+      <c r="P91">
+        <v>2.728313718840442</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>48</v>
+      </c>
+      <c r="R91">
+        <v>3.309419265488571</v>
+      </c>
+      <c r="S91">
+        <v>0.7155038724049491</v>
+      </c>
+      <c r="T91">
+        <v>15.30705324902608</v>
+      </c>
+      <c r="U91">
+        <v>1.531549889862875</v>
+      </c>
+      <c r="V91">
+        <v>0.1256335462018899</v>
+      </c>
+      <c r="Y91">
+        <v>0.5811539804444464</v>
+      </c>
+      <c r="Z91">
+        <v>331.9086412875165</v>
+      </c>
+      <c r="AA91">
+        <v>0.03099809921225616</v>
+      </c>
+      <c r="AD91">
+        <v>-0.01962586642447821</v>
+      </c>
+      <c r="AE91">
+        <v>0.757921675728828</v>
+      </c>
+      <c r="AF91">
+        <v>0.02310477793664775</v>
+      </c>
+      <c r="AG91">
+        <v>0.2889220518073117</v>
+      </c>
+      <c r="AH91">
+        <v>0.7680579011322347</v>
+      </c>
+    </row>
+    <row r="92" spans="1:39">
+      <c r="A92" t="s">
+        <v>154</v>
+      </c>
+      <c r="B92" t="s">
+        <v>85</v>
+      </c>
+      <c r="C92" t="s">
+        <v>149</v>
+      </c>
+      <c r="D92" t="s">
+        <v>41</v>
+      </c>
+      <c r="E92" t="b">
+        <v>0</v>
+      </c>
+      <c r="F92" t="s">
+        <v>107</v>
+      </c>
+      <c r="G92" t="s">
+        <v>43</v>
+      </c>
+      <c r="H92">
+        <v>354</v>
+      </c>
+      <c r="I92" t="s">
+        <v>87</v>
+      </c>
+      <c r="J92" t="s">
+        <v>88</v>
+      </c>
+      <c r="K92" t="s">
+        <v>89</v>
+      </c>
+      <c r="L92" t="s">
+        <v>82</v>
+      </c>
+      <c r="M92">
+        <v>-0.02594997392866997</v>
+      </c>
+      <c r="N92">
+        <v>0.071135629884542</v>
+      </c>
+      <c r="O92">
+        <v>-0.1653732465199434</v>
+      </c>
+      <c r="P92">
+        <v>0.1134732986626035</v>
+      </c>
+      <c r="Q92" t="s">
+        <v>48</v>
+      </c>
+      <c r="R92">
+        <v>0.974383832984651</v>
+      </c>
+      <c r="S92">
+        <v>0.8475772897675284</v>
+      </c>
+      <c r="T92">
+        <v>1.12016197867013</v>
+      </c>
+      <c r="U92">
+        <v>-0.3647957285370012</v>
+      </c>
+      <c r="V92">
+        <v>0.7152638938383014</v>
+      </c>
+      <c r="W92" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y92">
+        <v>1.47212996434032</v>
+      </c>
+      <c r="Z92">
+        <v>609.9411060192901</v>
+      </c>
+      <c r="AA92">
+        <v>0.002872421971886752</v>
+      </c>
+      <c r="AD92">
+        <v>0.06279222907713251</v>
+      </c>
+      <c r="AE92">
+        <v>0.003130964596513673</v>
+      </c>
+      <c r="AF92">
+        <v>0.08911545059792679</v>
+      </c>
+      <c r="AG92">
+        <v>0.02533783719221571</v>
+      </c>
+      <c r="AH92">
+        <v>0.0002418776573451797</v>
+      </c>
+      <c r="AI92">
+        <v>-0.009214017199138107</v>
+      </c>
+      <c r="AJ92">
+        <v>0.6048136069684058</v>
+      </c>
+      <c r="AK92">
+        <v>-0.01903187605963569</v>
+      </c>
+      <c r="AL92">
+        <v>0.6314828734756739</v>
+      </c>
+      <c r="AM92">
+        <v>0.3027195787835912</v>
+      </c>
+    </row>
+    <row r="93" spans="1:39">
+      <c r="A93" t="s">
+        <v>154</v>
+      </c>
+      <c r="B93" t="s">
+        <v>90</v>
+      </c>
+      <c r="C93" t="s">
+        <v>149</v>
+      </c>
+      <c r="D93" t="s">
+        <v>41</v>
+      </c>
+      <c r="E93" t="b">
+        <v>0</v>
+      </c>
+      <c r="F93" t="s">
+        <v>107</v>
+      </c>
+      <c r="G93" t="s">
+        <v>43</v>
+      </c>
+      <c r="H93">
+        <v>354</v>
+      </c>
+      <c r="I93" t="s">
+        <v>91</v>
+      </c>
+      <c r="J93" t="s">
+        <v>92</v>
+      </c>
+      <c r="K93" t="s">
+        <v>93</v>
+      </c>
+      <c r="L93" t="s">
+        <v>94</v>
+      </c>
+      <c r="M93">
+        <v>0.2638673268239927</v>
+      </c>
+      <c r="N93">
+        <v>0.2083313688377325</v>
+      </c>
+      <c r="O93">
+        <v>-0.1444546529478929</v>
+      </c>
+      <c r="P93">
+        <v>0.6721893065958784</v>
+      </c>
+      <c r="Q93" t="s">
+        <v>48</v>
+      </c>
+      <c r="R93">
+        <v>1.301955450277158</v>
+      </c>
+      <c r="S93">
+        <v>0.8654941591219707</v>
+      </c>
+      <c r="T93">
+        <v>1.958520432103244</v>
+      </c>
+      <c r="U93">
+        <v>1.266575112025097</v>
+      </c>
+      <c r="V93">
+        <v>0.2053072561997599</v>
+      </c>
+      <c r="Y93">
+        <v>1.47212996434032</v>
+      </c>
+      <c r="Z93">
+        <v>609.9411060192901</v>
+      </c>
+      <c r="AA93">
+        <v>0.002872421971886752</v>
+      </c>
+      <c r="AD93">
+        <v>0.06279222907713251</v>
+      </c>
+      <c r="AE93">
+        <v>0.003130964596513673</v>
+      </c>
+      <c r="AF93">
+        <v>0.08911545059792679</v>
+      </c>
+      <c r="AG93">
+        <v>0.02533783719221571</v>
+      </c>
+      <c r="AH93">
+        <v>0.0002418776573451797</v>
+      </c>
+      <c r="AI93">
+        <v>-0.009214017199138107</v>
+      </c>
+      <c r="AJ93">
+        <v>0.6048136069684058</v>
+      </c>
+      <c r="AK93">
+        <v>-0.01903187605963569</v>
+      </c>
+      <c r="AL93">
+        <v>0.6314828734756739</v>
+      </c>
+      <c r="AM93">
+        <v>0.3027195787835912</v>
+      </c>
+    </row>
+    <row r="94" spans="1:39">
+      <c r="A94" t="s">
+        <v>154</v>
+      </c>
+      <c r="B94" t="s">
+        <v>90</v>
+      </c>
+      <c r="C94" t="s">
+        <v>149</v>
+      </c>
+      <c r="D94" t="s">
+        <v>41</v>
+      </c>
+      <c r="E94" t="b">
+        <v>0</v>
+      </c>
+      <c r="F94" t="s">
+        <v>107</v>
+      </c>
+      <c r="G94" t="s">
+        <v>43</v>
+      </c>
+      <c r="H94">
+        <v>354</v>
+      </c>
+      <c r="I94" t="s">
+        <v>95</v>
+      </c>
+      <c r="J94" t="s">
+        <v>96</v>
+      </c>
+      <c r="K94" t="s">
+        <v>97</v>
+      </c>
+      <c r="L94" t="s">
+        <v>94</v>
+      </c>
+      <c r="M94">
+        <v>0.2866787909467804</v>
+      </c>
+      <c r="N94">
+        <v>0.6186263489458452</v>
+      </c>
+      <c r="O94">
+        <v>-0.925806572874584</v>
+      </c>
+      <c r="P94">
+        <v>1.499164154768145</v>
+      </c>
+      <c r="Q94" t="s">
+        <v>48</v>
+      </c>
+      <c r="R94">
+        <v>1.331996295484824</v>
+      </c>
+      <c r="S94">
+        <v>0.3962117165374762</v>
+      </c>
+      <c r="T94">
+        <v>4.477944636999342</v>
+      </c>
+      <c r="U94">
+        <v>0.4634118663637399</v>
+      </c>
+      <c r="V94">
+        <v>0.6430691745964943</v>
+      </c>
+      <c r="Y94">
+        <v>1.47212996434032</v>
+      </c>
+      <c r="Z94">
+        <v>609.9411060192901</v>
+      </c>
+      <c r="AA94">
+        <v>0.002872421971886752</v>
+      </c>
+      <c r="AD94">
+        <v>0.06279222907713251</v>
+      </c>
+      <c r="AE94">
+        <v>0.003130964596513673</v>
+      </c>
+      <c r="AF94">
+        <v>0.08911545059792679</v>
+      </c>
+      <c r="AG94">
+        <v>0.02533783719221571</v>
+      </c>
+      <c r="AH94">
+        <v>0.0002418776573451797</v>
+      </c>
+      <c r="AI94">
+        <v>-0.009214017199138107</v>
+      </c>
+      <c r="AJ94">
+        <v>0.6048136069684058</v>
+      </c>
+      <c r="AK94">
+        <v>-0.01903187605963569</v>
+      </c>
+      <c r="AL94">
+        <v>0.6314828734756739</v>
+      </c>
+      <c r="AM94">
+        <v>0.3027195787835912</v>
+      </c>
+    </row>
+    <row r="95" spans="1:39">
+      <c r="A95" t="s">
+        <v>154</v>
+      </c>
+      <c r="B95" t="s">
+        <v>85</v>
+      </c>
+      <c r="C95" t="s">
+        <v>149</v>
+      </c>
+      <c r="D95" t="s">
+        <v>50</v>
+      </c>
+      <c r="E95" t="b">
+        <v>1</v>
+      </c>
+      <c r="F95" t="s">
+        <v>107</v>
+      </c>
+      <c r="G95" t="s">
+        <v>51</v>
+      </c>
+      <c r="H95">
+        <v>354</v>
+      </c>
+      <c r="I95" t="s">
+        <v>87</v>
+      </c>
+      <c r="J95" t="s">
+        <v>88</v>
+      </c>
+      <c r="K95" t="s">
+        <v>89</v>
+      </c>
+      <c r="L95" t="s">
+        <v>82</v>
+      </c>
+      <c r="M95">
+        <v>-0.04583810019367455</v>
+      </c>
+      <c r="N95">
+        <v>0.07567974050219441</v>
+      </c>
+      <c r="O95">
+        <v>-0.1941676659373128</v>
+      </c>
+      <c r="P95">
+        <v>0.1024914655499637</v>
+      </c>
+      <c r="Q95" t="s">
+        <v>48</v>
+      </c>
+      <c r="R95">
+        <v>0.9551965958166653</v>
+      </c>
+      <c r="S95">
+        <v>0.8235198164706661</v>
+      </c>
+      <c r="T95">
+        <v>1.107927846314607</v>
+      </c>
+      <c r="U95">
+        <v>-0.6056852189172799</v>
+      </c>
+      <c r="V95">
+        <v>0.5447238011190841</v>
+      </c>
+      <c r="W95" t="s">
+        <v>83</v>
+      </c>
+      <c r="X95" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z95">
+        <v>590.1943882673806</v>
+      </c>
+      <c r="AA95">
+        <v>0.003458868848606245</v>
+      </c>
+      <c r="AB95">
+        <v>14.4786245108509</v>
+      </c>
+      <c r="AC95">
+        <v>0.8435062336650891</v>
+      </c>
+      <c r="AD95">
+        <v>0.06279222907713251</v>
+      </c>
+      <c r="AE95">
+        <v>0.003130964596513673</v>
+      </c>
+      <c r="AF95">
+        <v>0.08911545059792679</v>
+      </c>
+      <c r="AG95">
+        <v>0.02533783719221571</v>
+      </c>
+      <c r="AH95">
+        <v>0.0002418776573451797</v>
+      </c>
+      <c r="AI95">
+        <v>-0.009214017199138107</v>
+      </c>
+      <c r="AJ95">
+        <v>0.6048136069684058</v>
+      </c>
+      <c r="AK95">
+        <v>-0.01903187605963569</v>
+      </c>
+      <c r="AL95">
+        <v>0.6314828734756739</v>
+      </c>
+      <c r="AM95">
+        <v>0.3027195787835912</v>
+      </c>
+    </row>
+    <row r="96" spans="1:39">
+      <c r="A96" t="s">
+        <v>154</v>
+      </c>
+      <c r="B96" t="s">
+        <v>90</v>
+      </c>
+      <c r="C96" t="s">
+        <v>149</v>
+      </c>
+      <c r="D96" t="s">
+        <v>50</v>
+      </c>
+      <c r="E96" t="b">
+        <v>1</v>
+      </c>
+      <c r="F96" t="s">
+        <v>107</v>
+      </c>
+      <c r="G96" t="s">
+        <v>51</v>
+      </c>
+      <c r="H96">
+        <v>354</v>
+      </c>
+      <c r="I96" t="s">
+        <v>91</v>
+      </c>
+      <c r="J96" t="s">
+        <v>92</v>
+      </c>
+      <c r="K96" t="s">
+        <v>93</v>
+      </c>
+      <c r="L96" t="s">
+        <v>94</v>
+      </c>
+      <c r="M96">
+        <v>0.1624220401044004</v>
+      </c>
+      <c r="N96">
+        <v>0.2231800658671059</v>
+      </c>
+      <c r="O96">
+        <v>-0.2750028510624042</v>
+      </c>
+      <c r="P96">
+        <v>0.5998469312712049</v>
+      </c>
+      <c r="Q96" t="s">
+        <v>48</v>
+      </c>
+      <c r="R96">
+        <v>1.17635660623559</v>
+      </c>
+      <c r="S96">
+        <v>0.7595699576405318</v>
+      </c>
+      <c r="T96">
+        <v>1.821839912327085</v>
+      </c>
+      <c r="U96">
+        <v>0.7277623092069329</v>
+      </c>
+      <c r="V96">
+        <v>0.4667591005103527</v>
+      </c>
+      <c r="Z96">
+        <v>590.1943882673806</v>
+      </c>
+      <c r="AA96">
+        <v>0.003458868848606245</v>
+      </c>
+      <c r="AB96">
+        <v>14.4786245108509</v>
+      </c>
+      <c r="AC96">
+        <v>0.8435062336650891</v>
+      </c>
+      <c r="AD96">
+        <v>0.06279222907713251</v>
+      </c>
+      <c r="AE96">
+        <v>0.003130964596513673</v>
+      </c>
+      <c r="AF96">
+        <v>0.08911545059792679</v>
+      </c>
+      <c r="AG96">
+        <v>0.02533783719221571</v>
+      </c>
+      <c r="AH96">
+        <v>0.0002418776573451797</v>
+      </c>
+      <c r="AI96">
+        <v>-0.009214017199138107</v>
+      </c>
+      <c r="AJ96">
+        <v>0.6048136069684058</v>
+      </c>
+      <c r="AK96">
+        <v>-0.01903187605963569</v>
+      </c>
+      <c r="AL96">
+        <v>0.6314828734756739</v>
+      </c>
+      <c r="AM96">
+        <v>0.3027195787835912</v>
+      </c>
+    </row>
+    <row r="97" spans="1:39">
+      <c r="A97" t="s">
+        <v>154</v>
+      </c>
+      <c r="B97" t="s">
+        <v>90</v>
+      </c>
+      <c r="C97" t="s">
+        <v>149</v>
+      </c>
+      <c r="D97" t="s">
+        <v>50</v>
+      </c>
+      <c r="E97" t="b">
+        <v>1</v>
+      </c>
+      <c r="F97" t="s">
+        <v>107</v>
+      </c>
+      <c r="G97" t="s">
+        <v>51</v>
+      </c>
+      <c r="H97">
+        <v>354</v>
+      </c>
+      <c r="I97" t="s">
+        <v>95</v>
+      </c>
+      <c r="J97" t="s">
+        <v>96</v>
+      </c>
+      <c r="K97" t="s">
+        <v>97</v>
+      </c>
+      <c r="L97" t="s">
+        <v>94</v>
+      </c>
+      <c r="M97">
+        <v>0.7849404605872226</v>
+      </c>
+      <c r="N97">
+        <v>0.6327445103324674</v>
+      </c>
+      <c r="O97">
+        <v>-0.4552159910798452</v>
+      </c>
+      <c r="P97">
+        <v>2.02509691225429</v>
+      </c>
+      <c r="Q97" t="s">
+        <v>48</v>
+      </c>
+      <c r="R97">
+        <v>2.192276409997295</v>
+      </c>
+      <c r="S97">
+        <v>0.6343109476446398</v>
+      </c>
+      <c r="T97">
+        <v>7.576845198205754</v>
+      </c>
+      <c r="U97">
+        <v>1.24053302362874</v>
+      </c>
+      <c r="V97">
+        <v>0.2147783074166748</v>
+      </c>
+      <c r="Z97">
+        <v>590.1943882673806</v>
+      </c>
+      <c r="AA97">
+        <v>0.003458868848606245</v>
+      </c>
+      <c r="AB97">
+        <v>14.4786245108509</v>
+      </c>
+      <c r="AC97">
+        <v>0.8435062336650891</v>
+      </c>
+      <c r="AD97">
+        <v>0.06279222907713251</v>
+      </c>
+      <c r="AE97">
+        <v>0.003130964596513673</v>
+      </c>
+      <c r="AF97">
+        <v>0.08911545059792679</v>
+      </c>
+      <c r="AG97">
+        <v>0.02533783719221571</v>
+      </c>
+      <c r="AH97">
+        <v>0.0002418776573451797</v>
+      </c>
+      <c r="AI97">
+        <v>-0.009214017199138107</v>
+      </c>
+      <c r="AJ97">
+        <v>0.6048136069684058</v>
+      </c>
+      <c r="AK97">
+        <v>-0.01903187605963569</v>
+      </c>
+      <c r="AL97">
+        <v>0.6314828734756739</v>
+      </c>
+      <c r="AM97">
+        <v>0.3027195787835912</v>
+      </c>
+    </row>
+    <row r="98" spans="1:39">
+      <c r="A98" t="s">
+        <v>155</v>
+      </c>
+      <c r="B98" t="s">
+        <v>100</v>
+      </c>
+      <c r="C98" t="s">
+        <v>149</v>
+      </c>
+      <c r="D98" t="s">
+        <v>41</v>
+      </c>
+      <c r="E98" t="b">
+        <v>1</v>
+      </c>
+      <c r="F98" t="s">
+        <v>101</v>
+      </c>
+      <c r="G98" t="s">
+        <v>43</v>
+      </c>
+      <c r="H98">
+        <v>374</v>
+      </c>
+      <c r="I98" t="s">
+        <v>156</v>
+      </c>
+      <c r="J98" t="s">
+        <v>157</v>
+      </c>
+      <c r="K98" t="s">
+        <v>158</v>
+      </c>
+      <c r="L98" t="s">
+        <v>159</v>
+      </c>
+      <c r="M98">
+        <v>0.5362889187684159</v>
+      </c>
+      <c r="N98">
+        <v>0.3518360020097002</v>
+      </c>
+      <c r="O98">
+        <v>-0.1532969736351585</v>
+      </c>
+      <c r="P98">
+        <v>1.22587481117199</v>
+      </c>
+      <c r="Q98" t="s">
+        <v>48</v>
+      </c>
+      <c r="R98">
+        <v>1.709650423251085</v>
+      </c>
+      <c r="S98">
+        <v>0.8578749177453875</v>
+      </c>
+      <c r="T98">
+        <v>3.407145388286216</v>
+      </c>
+      <c r="U98">
+        <v>1.52425822174284</v>
+      </c>
+      <c r="V98">
+        <v>0.1274442191029556</v>
+      </c>
+      <c r="W98" t="s">
+        <v>49</v>
+      </c>
+      <c r="X98" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y98">
+        <v>1.756930293317255</v>
+      </c>
+      <c r="Z98">
+        <v>630.1717340608834</v>
+      </c>
+      <c r="AA98">
+        <v>0.01264958433481189</v>
+      </c>
+      <c r="AD98">
+        <v>0.0002674869681268992</v>
+      </c>
+      <c r="AE98">
+        <v>0.4498676132664657</v>
+      </c>
+      <c r="AF98">
+        <v>-0.01008496105843576</v>
+      </c>
+      <c r="AG98">
+        <v>0.5618393027158205</v>
+      </c>
+      <c r="AH98">
+        <v>0.7296574749189193</v>
+      </c>
+    </row>
+    <row r="99" spans="1:39">
+      <c r="A99" t="s">
+        <v>155</v>
+      </c>
+      <c r="B99" t="s">
+        <v>100</v>
+      </c>
+      <c r="C99" t="s">
+        <v>149</v>
+      </c>
+      <c r="D99" t="s">
+        <v>41</v>
+      </c>
+      <c r="E99" t="b">
+        <v>1</v>
+      </c>
+      <c r="F99" t="s">
+        <v>101</v>
+      </c>
+      <c r="G99" t="s">
+        <v>43</v>
+      </c>
+      <c r="H99">
+        <v>374</v>
+      </c>
+      <c r="I99" t="s">
+        <v>160</v>
+      </c>
+      <c r="J99" t="s">
+        <v>161</v>
+      </c>
+      <c r="K99" t="s">
+        <v>162</v>
+      </c>
+      <c r="L99" t="s">
+        <v>159</v>
+      </c>
+      <c r="M99">
+        <v>0.8108087535731383</v>
+      </c>
+      <c r="N99">
+        <v>0.4495394725355707</v>
+      </c>
+      <c r="O99">
+        <v>-0.07027242222571284</v>
+      </c>
+      <c r="P99">
+        <v>1.691889929371989</v>
+      </c>
+      <c r="Q99" t="s">
+        <v>48</v>
+      </c>
+      <c r="R99">
+        <v>2.24972672564947</v>
+      </c>
+      <c r="S99">
+        <v>0.9321398497014234</v>
+      </c>
+      <c r="T99">
+        <v>5.429732825737121</v>
+      </c>
+      <c r="U99">
+        <v>1.803643068315834</v>
+      </c>
+      <c r="V99">
+        <v>0.07128727981577819</v>
+      </c>
+      <c r="W99" t="s">
+        <v>49</v>
+      </c>
+      <c r="X99" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y99">
+        <v>1.756930293317255</v>
+      </c>
+      <c r="Z99">
+        <v>630.1717340608834</v>
+      </c>
+      <c r="AA99">
+        <v>0.01264958433481189</v>
+      </c>
+      <c r="AD99">
+        <v>0.0002674869681268992</v>
+      </c>
+      <c r="AE99">
+        <v>0.4498676132664657</v>
+      </c>
+      <c r="AF99">
+        <v>-0.01008496105843576</v>
+      </c>
+      <c r="AG99">
+        <v>0.5618393027158205</v>
+      </c>
+      <c r="AH99">
+        <v>0.7296574749189193</v>
+      </c>
+    </row>
+    <row r="100" spans="1:39">
+      <c r="A100" t="s">
+        <v>155</v>
+      </c>
+      <c r="B100" t="s">
+        <v>100</v>
+      </c>
+      <c r="C100" t="s">
+        <v>149</v>
+      </c>
+      <c r="D100" t="s">
+        <v>41</v>
+      </c>
+      <c r="E100" t="b">
+        <v>1</v>
+      </c>
+      <c r="F100" t="s">
+        <v>101</v>
+      </c>
+      <c r="G100" t="s">
+        <v>43</v>
+      </c>
+      <c r="H100">
+        <v>374</v>
+      </c>
+      <c r="I100" t="s">
+        <v>163</v>
+      </c>
+      <c r="J100" t="s">
+        <v>164</v>
+      </c>
+      <c r="K100" t="s">
+        <v>165</v>
+      </c>
+      <c r="L100" t="s">
+        <v>159</v>
+      </c>
+      <c r="M100">
+        <v>1.917115479880704</v>
+      </c>
+      <c r="N100">
+        <v>0.6820965625152101</v>
+      </c>
+      <c r="O100">
+        <v>0.5802307833723186</v>
+      </c>
+      <c r="P100">
+        <v>3.254000176389089</v>
+      </c>
+      <c r="Q100" t="s">
+        <v>48</v>
+      </c>
+      <c r="R100">
+        <v>6.801311626831928</v>
+      </c>
+      <c r="S100">
+        <v>1.786450666288937</v>
+      </c>
+      <c r="T100">
+        <v>25.89371244232138</v>
+      </c>
+      <c r="U100">
+        <v>2.810621816962981</v>
+      </c>
+      <c r="V100">
+        <v>0.004944586716896902</v>
+      </c>
+      <c r="W100" t="s">
+        <v>49</v>
+      </c>
+      <c r="X100" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y100">
+        <v>1.756930293317255</v>
+      </c>
+      <c r="Z100">
+        <v>630.1717340608834</v>
+      </c>
+      <c r="AA100">
+        <v>0.01264958433481189</v>
+      </c>
+      <c r="AD100">
+        <v>0.0002674869681268992</v>
+      </c>
+      <c r="AE100">
+        <v>0.4498676132664657</v>
+      </c>
+      <c r="AF100">
+        <v>-0.01008496105843576</v>
+      </c>
+      <c r="AG100">
+        <v>0.5618393027158205</v>
+      </c>
+      <c r="AH100">
+        <v>0.7296574749189193</v>
+      </c>
+    </row>
+    <row r="101" spans="1:39">
+      <c r="A101" t="s">
+        <v>166</v>
+      </c>
+      <c r="B101" t="s">
+        <v>100</v>
+      </c>
+      <c r="C101" t="s">
+        <v>149</v>
+      </c>
+      <c r="D101" t="s">
+        <v>41</v>
+      </c>
+      <c r="E101" t="b">
+        <v>1</v>
+      </c>
+      <c r="F101" t="s">
+        <v>107</v>
+      </c>
+      <c r="G101" t="s">
+        <v>108</v>
+      </c>
+      <c r="H101">
+        <v>365</v>
+      </c>
+      <c r="I101" t="s">
+        <v>156</v>
+      </c>
+      <c r="J101" t="s">
+        <v>157</v>
+      </c>
+      <c r="K101" t="s">
+        <v>158</v>
+      </c>
+      <c r="L101" t="s">
+        <v>159</v>
+      </c>
+      <c r="M101">
+        <v>0.02339300169489493</v>
+      </c>
+      <c r="N101">
+        <v>0.3361258776673434</v>
+      </c>
+      <c r="O101">
+        <v>-0.6354016128050141</v>
+      </c>
+      <c r="P101">
+        <v>0.6821876161948038</v>
+      </c>
+      <c r="Q101" t="s">
+        <v>48</v>
+      </c>
+      <c r="R101">
+        <v>1.02366876406387</v>
+      </c>
+      <c r="S101">
+        <v>0.5297227021713093</v>
+      </c>
+      <c r="T101">
+        <v>1.978200545728484</v>
+      </c>
+      <c r="U101">
+        <v>0.06959595570932652</v>
+      </c>
+      <c r="V101">
+        <v>0.9445152560135034</v>
+      </c>
+      <c r="W101" t="s">
+        <v>49</v>
+      </c>
+      <c r="X101" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z101">
+        <v>598.6893345329158</v>
+      </c>
+      <c r="AA101">
+        <v>0.01167136924742329</v>
+      </c>
+      <c r="AD101">
+        <v>0.0005963141209567455</v>
+      </c>
+      <c r="AE101">
+        <v>0.4437640765909484</v>
+      </c>
+      <c r="AF101">
+        <v>0.0272874657852239</v>
+      </c>
+      <c r="AG101">
+        <v>0.2545027342663077</v>
+      </c>
+      <c r="AH101">
+        <v>0.3469882281035148</v>
+      </c>
+    </row>
+    <row r="102" spans="1:39">
+      <c r="A102" t="s">
+        <v>166</v>
+      </c>
+      <c r="B102" t="s">
+        <v>100</v>
+      </c>
+      <c r="C102" t="s">
+        <v>149</v>
+      </c>
+      <c r="D102" t="s">
+        <v>41</v>
+      </c>
+      <c r="E102" t="b">
+        <v>1</v>
+      </c>
+      <c r="F102" t="s">
+        <v>107</v>
+      </c>
+      <c r="G102" t="s">
+        <v>108</v>
+      </c>
+      <c r="H102">
+        <v>365</v>
+      </c>
+      <c r="I102" t="s">
+        <v>160</v>
+      </c>
+      <c r="J102" t="s">
+        <v>161</v>
+      </c>
+      <c r="K102" t="s">
+        <v>162</v>
+      </c>
+      <c r="L102" t="s">
+        <v>159</v>
+      </c>
+      <c r="M102">
+        <v>0.375905230575814</v>
+      </c>
+      <c r="N102">
+        <v>0.4403294238167053</v>
+      </c>
+      <c r="O102">
+        <v>-0.4871245814382016</v>
+      </c>
+      <c r="P102">
+        <v>1.23893504258983</v>
+      </c>
+      <c r="Q102" t="s">
+        <v>48</v>
+      </c>
+      <c r="R102">
+        <v>1.456309113655008</v>
+      </c>
+      <c r="S102">
+        <v>0.6143904865261695</v>
+      </c>
+      <c r="T102">
+        <v>3.451935342466113</v>
+      </c>
+      <c r="U102">
+        <v>0.8536909192157257</v>
+      </c>
+      <c r="V102">
+        <v>0.3932762669267992</v>
+      </c>
+      <c r="W102" t="s">
+        <v>49</v>
+      </c>
+      <c r="X102" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z102">
+        <v>598.6893345329158</v>
+      </c>
+      <c r="AA102">
+        <v>0.01167136924742329</v>
+      </c>
+      <c r="AD102">
+        <v>0.0005963141209567455</v>
+      </c>
+      <c r="AE102">
+        <v>0.4437640765909484</v>
+      </c>
+      <c r="AF102">
+        <v>0.0272874657852239</v>
+      </c>
+      <c r="AG102">
+        <v>0.2545027342663077</v>
+      </c>
+      <c r="AH102">
+        <v>0.3469882281035148</v>
+      </c>
+    </row>
+    <row r="103" spans="1:39">
+      <c r="A103" t="s">
+        <v>166</v>
+      </c>
+      <c r="B103" t="s">
+        <v>100</v>
+      </c>
+      <c r="C103" t="s">
+        <v>149</v>
+      </c>
+      <c r="D103" t="s">
+        <v>41</v>
+      </c>
+      <c r="E103" t="b">
+        <v>1</v>
+      </c>
+      <c r="F103" t="s">
+        <v>107</v>
+      </c>
+      <c r="G103" t="s">
+        <v>108</v>
+      </c>
+      <c r="H103">
+        <v>365</v>
+      </c>
+      <c r="I103" t="s">
+        <v>163</v>
+      </c>
+      <c r="J103" t="s">
+        <v>164</v>
+      </c>
+      <c r="K103" t="s">
+        <v>165</v>
+      </c>
+      <c r="L103" t="s">
+        <v>159</v>
+      </c>
+      <c r="M103">
+        <v>1.461351208757332</v>
+      </c>
+      <c r="N103">
+        <v>0.6502888108778544</v>
+      </c>
+      <c r="O103">
+        <v>0.186808559887359</v>
+      </c>
+      <c r="P103">
+        <v>2.735893857627305</v>
+      </c>
+      <c r="Q103" t="s">
+        <v>48</v>
+      </c>
+      <c r="R103">
+        <v>4.311781711175008</v>
+      </c>
+      <c r="S103">
+        <v>1.20539650171797</v>
+      </c>
+      <c r="T103">
+        <v>15.4235237105186</v>
+      </c>
+      <c r="U103">
+        <v>2.247234127840194</v>
+      </c>
+      <c r="V103">
+        <v>0.02462506818123131</v>
+      </c>
+      <c r="W103" t="s">
+        <v>49</v>
+      </c>
+      <c r="X103" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z103">
+        <v>598.6893345329158</v>
+      </c>
+      <c r="AA103">
+        <v>0.01167136924742329</v>
+      </c>
+      <c r="AD103">
+        <v>0.0005963141209567455</v>
+      </c>
+      <c r="AE103">
+        <v>0.4437640765909484</v>
+      </c>
+      <c r="AF103">
+        <v>0.0272874657852239</v>
+      </c>
+      <c r="AG103">
+        <v>0.2545027342663077</v>
+      </c>
+      <c r="AH103">
+        <v>0.3469882281035148</v>
+      </c>
+    </row>
+    <row r="104" spans="1:39">
+      <c r="A104" t="s">
+        <v>166</v>
+      </c>
+      <c r="B104" t="s">
+        <v>90</v>
+      </c>
+      <c r="C104" t="s">
+        <v>149</v>
+      </c>
+      <c r="D104" t="s">
+        <v>41</v>
+      </c>
+      <c r="E104" t="b">
+        <v>1</v>
+      </c>
+      <c r="F104" t="s">
+        <v>107</v>
+      </c>
+      <c r="G104" t="s">
+        <v>108</v>
+      </c>
+      <c r="H104">
+        <v>365</v>
+      </c>
+      <c r="I104" t="s">
+        <v>91</v>
+      </c>
+      <c r="J104" t="s">
+        <v>92</v>
+      </c>
+      <c r="K104" t="s">
+        <v>93</v>
+      </c>
+      <c r="L104" t="s">
+        <v>94</v>
+      </c>
+      <c r="M104">
+        <v>0.03702360929177987</v>
+      </c>
+      <c r="N104">
+        <v>0.2142450110489068</v>
+      </c>
+      <c r="O104">
+        <v>-0.3828888962314632</v>
+      </c>
+      <c r="P104">
+        <v>0.456936114815023</v>
+      </c>
+      <c r="Q104" t="s">
+        <v>48</v>
+      </c>
+      <c r="R104">
+        <v>1.037717520324671</v>
+      </c>
+      <c r="S104">
+        <v>0.6818886554768594</v>
+      </c>
+      <c r="T104">
+        <v>1.579227991754333</v>
+      </c>
+      <c r="U104">
+        <v>0.1728096682882773</v>
+      </c>
+      <c r="V104">
+        <v>0.8628010371884052</v>
+      </c>
+      <c r="Z104">
+        <v>598.6893345329158</v>
+      </c>
+      <c r="AA104">
+        <v>0.01167136924742329</v>
+      </c>
+      <c r="AD104">
+        <v>0.0005963141209567455</v>
+      </c>
+      <c r="AE104">
+        <v>0.4437640765909484</v>
+      </c>
+      <c r="AF104">
+        <v>0.0272874657852239</v>
+      </c>
+      <c r="AG104">
+        <v>0.2545027342663077</v>
+      </c>
+      <c r="AH104">
+        <v>0.3469882281035148</v>
+      </c>
+    </row>
+    <row r="105" spans="1:39">
+      <c r="A105" t="s">
+        <v>166</v>
+      </c>
+      <c r="B105" t="s">
+        <v>90</v>
+      </c>
+      <c r="C105" t="s">
+        <v>149</v>
+      </c>
+      <c r="D105" t="s">
+        <v>41</v>
+      </c>
+      <c r="E105" t="b">
+        <v>1</v>
+      </c>
+      <c r="F105" t="s">
+        <v>107</v>
+      </c>
+      <c r="G105" t="s">
+        <v>108</v>
+      </c>
+      <c r="H105">
+        <v>365</v>
+      </c>
+      <c r="I105" t="s">
+        <v>95</v>
+      </c>
+      <c r="J105" t="s">
+        <v>96</v>
+      </c>
+      <c r="K105" t="s">
+        <v>97</v>
+      </c>
+      <c r="L105" t="s">
+        <v>94</v>
+      </c>
+      <c r="M105">
+        <v>0.7978184222164202</v>
+      </c>
+      <c r="N105">
+        <v>0.6932058924998694</v>
+      </c>
+      <c r="O105">
+        <v>-0.5608401609542679</v>
+      </c>
+      <c r="P105">
+        <v>2.156477005387108</v>
+      </c>
+      <c r="Q105" t="s">
+        <v>48</v>
+      </c>
+      <c r="R105">
+        <v>2.220691029985341</v>
+      </c>
+      <c r="S105">
+        <v>0.5707293578399918</v>
+      </c>
+      <c r="T105">
+        <v>8.640643034942544</v>
+      </c>
+      <c r="U105">
+        <v>1.150911195141883</v>
+      </c>
+      <c r="V105">
+        <v>0.2497687716340106</v>
+      </c>
+      <c r="Z105">
+        <v>598.6893345329158</v>
+      </c>
+      <c r="AA105">
+        <v>0.01167136924742329</v>
+      </c>
+      <c r="AD105">
+        <v>0.0005963141209567455</v>
+      </c>
+      <c r="AE105">
+        <v>0.4437640765909484</v>
+      </c>
+      <c r="AF105">
+        <v>0.0272874657852239</v>
+      </c>
+      <c r="AG105">
+        <v>0.2545027342663077</v>
+      </c>
+      <c r="AH105">
+        <v>0.3469882281035148</v>
+      </c>
+    </row>
+    <row r="106" spans="1:39">
+      <c r="A106" t="s">
+        <v>167</v>
+      </c>
+      <c r="B106" t="s">
+        <v>110</v>
+      </c>
+      <c r="C106" t="s">
+        <v>149</v>
+      </c>
+      <c r="D106" t="s">
+        <v>41</v>
+      </c>
+      <c r="E106" t="b">
+        <v>1</v>
+      </c>
+      <c r="F106" t="s">
+        <v>42</v>
+      </c>
+      <c r="G106" t="s">
+        <v>43</v>
+      </c>
+      <c r="H106">
+        <v>226</v>
+      </c>
+      <c r="I106" t="s">
+        <v>113</v>
+      </c>
+      <c r="J106" t="s">
+        <v>114</v>
+      </c>
+      <c r="K106" t="s">
+        <v>115</v>
+      </c>
+      <c r="L106" t="s">
+        <v>116</v>
+      </c>
+      <c r="M106">
+        <v>0.4204831929660624</v>
+      </c>
+      <c r="N106">
+        <v>0.1319708336146649</v>
+      </c>
+      <c r="O106">
+        <v>0.1618251120715914</v>
+      </c>
+      <c r="P106">
+        <v>0.6791412738605334</v>
+      </c>
+      <c r="Q106" t="s">
+        <v>48</v>
+      </c>
+      <c r="R106">
+        <v>1.52269713443587</v>
+      </c>
+      <c r="S106">
+        <v>1.175654615540555</v>
+      </c>
+      <c r="T106">
+        <v>1.972183439396558</v>
+      </c>
+      <c r="U106">
+        <v>3.18618274545276</v>
+      </c>
+      <c r="V106">
+        <v>0.001441635039864584</v>
+      </c>
+      <c r="W106" t="s">
+        <v>49</v>
+      </c>
+      <c r="X106" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y106">
+        <v>1.847804844795774</v>
+      </c>
+      <c r="Z106">
+        <v>619.3403886128827</v>
+      </c>
+      <c r="AA106">
+        <v>0.02913853765991992</v>
+      </c>
+      <c r="AD106">
+        <v>-0.02104406814582626</v>
+      </c>
+      <c r="AE106">
+        <v>0.7130097650909896</v>
+      </c>
+      <c r="AF106">
+        <v>0.05664179320021405</v>
+      </c>
+      <c r="AG106">
+        <v>0.1908990300697498</v>
+      </c>
+      <c r="AH106">
+        <v>0.2595164925583584</v>
+      </c>
+    </row>
+    <row r="107" spans="1:39">
+      <c r="A107" t="s">
+        <v>167</v>
+      </c>
+      <c r="B107" t="s">
+        <v>120</v>
+      </c>
+      <c r="C107" t="s">
+        <v>149</v>
+      </c>
+      <c r="D107" t="s">
+        <v>41</v>
+      </c>
+      <c r="E107" t="b">
+        <v>1</v>
+      </c>
+      <c r="F107" t="s">
+        <v>42</v>
+      </c>
+      <c r="G107" t="s">
+        <v>43</v>
+      </c>
+      <c r="H107">
+        <v>226</v>
+      </c>
+      <c r="I107" t="s">
+        <v>121</v>
+      </c>
+      <c r="J107" t="s">
+        <v>122</v>
+      </c>
+      <c r="K107" t="s">
+        <v>123</v>
+      </c>
+      <c r="L107" t="s">
+        <v>124</v>
+      </c>
+      <c r="M107">
+        <v>-0.1845274916284873</v>
+      </c>
+      <c r="N107">
+        <v>0.05349148703698052</v>
+      </c>
+      <c r="O107">
+        <v>-0.2893688797004603</v>
+      </c>
+      <c r="P107">
+        <v>-0.07968610355651437</v>
+      </c>
+      <c r="Q107" t="s">
+        <v>48</v>
+      </c>
+      <c r="R107">
+        <v>0.8314970803763607</v>
+      </c>
+      <c r="S107">
+        <v>0.7487359609583156</v>
+      </c>
+      <c r="T107">
+        <v>0.9234061548072267</v>
+      </c>
+      <c r="U107">
+        <v>-3.449660905873061</v>
+      </c>
+      <c r="V107">
+        <v>0.0005612911158422043</v>
+      </c>
+      <c r="W107" t="s">
+        <v>68</v>
+      </c>
+      <c r="X107" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y107">
+        <v>1.847804844795774</v>
+      </c>
+      <c r="Z107">
+        <v>619.3403886128827</v>
+      </c>
+      <c r="AA107">
+        <v>0.02913853765991992</v>
+      </c>
+      <c r="AD107">
+        <v>-0.02104406814582626</v>
+      </c>
+      <c r="AE107">
+        <v>0.7130097650909896</v>
+      </c>
+      <c r="AF107">
+        <v>0.05664179320021405</v>
+      </c>
+      <c r="AG107">
+        <v>0.1908990300697498</v>
+      </c>
+      <c r="AH107">
+        <v>0.2595164925583584</v>
+      </c>
+    </row>
+    <row r="108" spans="1:39">
+      <c r="A108" t="s">
+        <v>168</v>
+      </c>
+      <c r="B108" t="s">
+        <v>110</v>
+      </c>
+      <c r="C108" t="s">
+        <v>149</v>
+      </c>
+      <c r="D108" t="s">
+        <v>41</v>
+      </c>
+      <c r="E108" t="b">
+        <v>1</v>
+      </c>
+      <c r="F108" t="s">
+        <v>42</v>
+      </c>
+      <c r="G108" t="s">
+        <v>43</v>
+      </c>
+      <c r="H108">
+        <v>202</v>
+      </c>
+      <c r="I108" t="s">
+        <v>113</v>
+      </c>
+      <c r="J108" t="s">
+        <v>114</v>
+      </c>
+      <c r="K108" t="s">
+        <v>115</v>
+      </c>
+      <c r="L108" t="s">
+        <v>116</v>
+      </c>
+      <c r="M108">
+        <v>0.4140782800973458</v>
+      </c>
+      <c r="N108">
+        <v>0.1321062908742811</v>
+      </c>
+      <c r="O108">
+        <v>0.1551547078525826</v>
+      </c>
+      <c r="P108">
+        <v>0.673001852342109</v>
+      </c>
+      <c r="Q108" t="s">
+        <v>48</v>
+      </c>
+      <c r="R108">
+        <v>1.512975558122901</v>
+      </c>
+      <c r="S108">
+        <v>1.167838620935225</v>
+      </c>
+      <c r="T108">
+        <v>1.960112466261954</v>
+      </c>
+      <c r="U108">
+        <v>3.134432715936316</v>
+      </c>
+      <c r="V108">
+        <v>0.001721867365777989</v>
+      </c>
+      <c r="W108" t="s">
+        <v>49</v>
+      </c>
+      <c r="X108" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y108">
+        <v>2.055689691353061</v>
+      </c>
+      <c r="Z108">
+        <v>583.4274508460501</v>
+      </c>
+      <c r="AA108">
+        <v>0.0268258891904074</v>
+      </c>
+      <c r="AD108">
+        <v>-0.04440392055852355</v>
+      </c>
+      <c r="AE108">
+        <v>0.8971384949822991</v>
+      </c>
+      <c r="AF108">
+        <v>0.03803659139362264</v>
+      </c>
+      <c r="AG108">
+        <v>0.2753145220809197</v>
+      </c>
+      <c r="AH108">
+        <v>0.4702112881795306</v>
+      </c>
+    </row>
+    <row r="109" spans="1:39">
+      <c r="A109" t="s">
+        <v>168</v>
+      </c>
+      <c r="B109" t="s">
+        <v>120</v>
+      </c>
+      <c r="C109" t="s">
+        <v>149</v>
+      </c>
+      <c r="D109" t="s">
+        <v>41</v>
+      </c>
+      <c r="E109" t="b">
+        <v>1</v>
+      </c>
+      <c r="F109" t="s">
+        <v>42</v>
+      </c>
+      <c r="G109" t="s">
+        <v>43</v>
+      </c>
+      <c r="H109">
+        <v>202</v>
+      </c>
+      <c r="I109" t="s">
+        <v>121</v>
+      </c>
+      <c r="J109" t="s">
+        <v>122</v>
+      </c>
+      <c r="K109" t="s">
+        <v>123</v>
+      </c>
+      <c r="L109" t="s">
+        <v>124</v>
+      </c>
+      <c r="M109">
+        <v>-0.1659273085960489</v>
+      </c>
+      <c r="N109">
+        <v>0.05353266861820654</v>
+      </c>
+      <c r="O109">
+        <v>-0.2708494110840513</v>
+      </c>
+      <c r="P109">
+        <v>-0.06100520610804655</v>
+      </c>
+      <c r="Q109" t="s">
+        <v>48</v>
+      </c>
+      <c r="R109">
+        <v>0.8471078094073418</v>
+      </c>
+      <c r="S109">
+        <v>0.7627313466439131</v>
+      </c>
+      <c r="T109">
+        <v>0.9408183417613205</v>
+      </c>
+      <c r="U109">
+        <v>-3.099552345866367</v>
+      </c>
+      <c r="V109">
+        <v>0.00193813326680686</v>
+      </c>
+      <c r="W109" t="s">
+        <v>68</v>
+      </c>
+      <c r="X109" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y109">
+        <v>2.055689691353061</v>
+      </c>
+      <c r="Z109">
+        <v>583.4274508460501</v>
+      </c>
+      <c r="AA109">
+        <v>0.0268258891904074</v>
+      </c>
+      <c r="AD109">
+        <v>-0.04440392055852355</v>
+      </c>
+      <c r="AE109">
+        <v>0.8971384949822991</v>
+      </c>
+      <c r="AF109">
+        <v>0.03803659139362264</v>
+      </c>
+      <c r="AG109">
+        <v>0.2753145220809197</v>
+      </c>
+      <c r="AH109">
+        <v>0.4702112881795306</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>